<commit_message>
fix: exchange corpus metadata xlsx
</commit_message>
<xml_diff>
--- a/data/metadata/corpus_metadata/corpus_metadata.xlsx
+++ b/data/metadata/corpus_metadata/corpus_metadata.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/deryademir/Documents/QUADRIGA/sfb_repository/data/metadata/corpus_metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B10DFDB-38F3-4045-9BF5-D92E5E390DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F58A58A-E5CA-C541-83B5-38857B4E8507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="23260" windowHeight="12460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Korpusmetadaten" sheetId="1" r:id="rId1"/>
+    <sheet name="corpus metadata" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -2908,7 +2908,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2921,7 +2921,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -12989,7 +12989,7 @@
       <formula>60</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:N226" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
       <formula2>0</formula2>
@@ -12998,26 +12998,15 @@
       <formula1>"Destabilization / Restabilization,Escalation / de-escalation,Disruptive scaling,Non-linear temporalities,Post-anthropocentric reperspectivations,Unintended Consequences,Collision,N/A,"</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D226" xr:uid="{00000000-0002-0000-0000-000002000000}">
+      <formula1>#REF!</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
-          <x14:formula1>
-            <xm:f>#REF!</xm:f>
-          </x14:formula1>
-          <x14:formula2>
-            <xm:f>0</xm:f>
-          </x14:formula2>
-          <xm:sqref>D2:D226</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
</xml_diff>